<commit_message>
slider new 2 ao 3ra vez y otros ajustes
</commit_message>
<xml_diff>
--- a/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2_15-10-2026.xlsx
+++ b/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2_15-10-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sgantolin\BiscaytikApp_node-modules-incluido\src\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD4E200-275A-43C2-B321-B9CF901C8A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6676DE-052C-4BF0-98D8-190CF8C7583E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="274">
   <si>
     <t>HITO</t>
   </si>
@@ -701,9 +701,6 @@
     <t>Condicionado. 1 ejem para todos los tipos</t>
   </si>
   <si>
-    <t xml:space="preserve">3.1 HOME </t>
-  </si>
-  <si>
     <t>validación contenidos</t>
   </si>
   <si>
@@ -782,12 +779,6 @@
     <t>En curso. No final. Fase 2</t>
   </si>
   <si>
-    <t>Suma y links (15/10/2026)</t>
-  </si>
-  <si>
-    <t>Suma y links</t>
-  </si>
-  <si>
     <t>85% Finalizado.  Ajustes css</t>
   </si>
   <si>
@@ -846,6 +837,30 @@
   </si>
   <si>
     <t>80% Finalizado. 1ra prueba hecha.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+I de información es un tooltip https://getbootstrap.com/docs/5.0/components/tooltips/ cualquier cosa nos comentáis pues tenemos el código en local
+La i he visto que tenía una BKTT-Icon dentro de otro BKTT-Icon. El padre debería ser BKTT-Button btn btn-link. I si el icono de dentro es &lt;i class="fa-regular fa-info"&gt;&lt;/i&gt; en vez del cicle fenomenal
+Las a's que entiendo que son los botones de CTA, deberían de tener la siguiente class BKTT-Button btn btn-primary. Sobre todo BKTT-Button</t>
+  </si>
+  <si>
+    <t>Muy dificil rojoy media amarillo</t>
+  </si>
+  <si>
+    <t>3.1 HOME http://turi.santurtzi.com/es-es/Paginas/Default2.aspx</t>
+  </si>
+  <si>
+    <t>SUMMARYLINKSLIDER2026</t>
+  </si>
+  <si>
+    <t>SUMMARYLINK2026</t>
+  </si>
+  <si>
+    <t>SUMMARYLINKSLIDER2026 (15/10/2026)</t>
+  </si>
+  <si>
+    <t>SUMMARYLINK2026 (15/10/2026)</t>
   </si>
 </sst>
 </file>
@@ -1016,7 +1031,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1149,6 +1164,12 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1164,7 +1185,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1330,6 +1351,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1641,7 +1665,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AI125"/>
+  <dimension ref="A1:AL126"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" outlineLevelRow="2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.33203125" style="49" customWidth="1"/>
@@ -1667,10 +1691,11 @@
     <col min="31" max="31" width="17.5546875" style="19" customWidth="1"/>
     <col min="32" max="32" width="12.88671875" style="19" customWidth="1"/>
     <col min="33" max="33" width="18.44140625" customWidth="1"/>
+    <col min="36" max="36" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="22.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:35" ht="216" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:38" ht="22.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:38" ht="216" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1757,7 +1782,7 @@
         <v>179</v>
       </c>
       <c r="AD2" s="35" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AE2" s="35" t="s">
         <v>180</v>
@@ -1766,7 +1791,7 @@
         <v>179</v>
       </c>
       <c r="AG2" s="35" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="AH2" s="35" t="s">
         <v>180</v>
@@ -1774,8 +1799,17 @@
       <c r="AI2" s="35" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="3" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ2" s="35" t="s">
+        <v>250</v>
+      </c>
+      <c r="AK2" s="35" t="s">
+        <v>180</v>
+      </c>
+      <c r="AL2" s="35" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A3" s="50">
         <v>0</v>
       </c>
@@ -1819,8 +1853,13 @@
       </c>
       <c r="AH3" s="19"/>
       <c r="AI3" s="19"/>
-    </row>
-    <row r="4" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ3" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK3" s="19"/>
+      <c r="AL3" s="19"/>
+    </row>
+    <row r="4" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D4" s="30" t="s">
         <v>13</v>
       </c>
@@ -1845,8 +1884,11 @@
       <c r="AG4" s="19"/>
       <c r="AH4" s="19"/>
       <c r="AI4" s="19"/>
-    </row>
-    <row r="5" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ4" s="19"/>
+      <c r="AK4" s="19"/>
+      <c r="AL4" s="19"/>
+    </row>
+    <row r="5" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D5" s="19" t="s">
         <v>16</v>
       </c>
@@ -1857,8 +1899,11 @@
       <c r="AG5" s="19"/>
       <c r="AH5" s="19"/>
       <c r="AI5" s="19"/>
-    </row>
-    <row r="6" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ5" s="19"/>
+      <c r="AK5" s="19"/>
+      <c r="AL5" s="19"/>
+    </row>
+    <row r="6" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D6" s="30" t="s">
         <v>17</v>
       </c>
@@ -1883,8 +1928,11 @@
       <c r="AG6" s="19"/>
       <c r="AH6" s="19"/>
       <c r="AI6" s="19"/>
-    </row>
-    <row r="7" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ6" s="19"/>
+      <c r="AK6" s="19"/>
+      <c r="AL6" s="19"/>
+    </row>
+    <row r="7" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D7" s="19" t="s">
         <v>20</v>
       </c>
@@ -1895,8 +1943,11 @@
       <c r="AG7" s="19"/>
       <c r="AH7" s="19"/>
       <c r="AI7" s="19"/>
-    </row>
-    <row r="8" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ7" s="19"/>
+      <c r="AK7" s="19"/>
+      <c r="AL7" s="19"/>
+    </row>
+    <row r="8" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D8" s="31" t="s">
         <v>21</v>
       </c>
@@ -1921,8 +1972,11 @@
       <c r="AG8" s="19"/>
       <c r="AH8" s="19"/>
       <c r="AI8" s="19"/>
-    </row>
-    <row r="9" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ8" s="19"/>
+      <c r="AK8" s="19"/>
+      <c r="AL8" s="19"/>
+    </row>
+    <row r="9" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D9" s="19" t="s">
         <v>22</v>
       </c>
@@ -1933,8 +1987,11 @@
       <c r="AG9" s="19"/>
       <c r="AH9" s="19"/>
       <c r="AI9" s="19"/>
-    </row>
-    <row r="10" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ9" s="19"/>
+      <c r="AK9" s="19"/>
+      <c r="AL9" s="19"/>
+    </row>
+    <row r="10" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A10" s="50">
         <v>1</v>
       </c>
@@ -1974,8 +2031,11 @@
       <c r="AG10" s="19"/>
       <c r="AH10" s="19"/>
       <c r="AI10" s="19"/>
-    </row>
-    <row r="11" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ10" s="19"/>
+      <c r="AK10" s="19"/>
+      <c r="AL10" s="19"/>
+    </row>
+    <row r="11" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A11" s="30" t="s">
         <v>26</v>
       </c>
@@ -2020,8 +2080,13 @@
       </c>
       <c r="AH11" s="19"/>
       <c r="AI11" s="19"/>
-    </row>
-    <row r="12" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ11" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK11" s="19"/>
+      <c r="AL11" s="19"/>
+    </row>
+    <row r="12" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>30</v>
       </c>
@@ -2041,8 +2106,11 @@
       <c r="AG12" s="19"/>
       <c r="AH12" s="19"/>
       <c r="AI12" s="19"/>
-    </row>
-    <row r="13" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ12" s="19"/>
+      <c r="AK12" s="19"/>
+      <c r="AL12" s="19"/>
+    </row>
+    <row r="13" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
         <v>31</v>
       </c>
@@ -2062,8 +2130,11 @@
       <c r="AG13" s="19"/>
       <c r="AH13" s="19"/>
       <c r="AI13" s="19"/>
-    </row>
-    <row r="14" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ13" s="19"/>
+      <c r="AK13" s="19"/>
+      <c r="AL13" s="19"/>
+    </row>
+    <row r="14" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>32</v>
       </c>
@@ -2083,8 +2154,11 @@
       <c r="AG14" s="19"/>
       <c r="AH14" s="19"/>
       <c r="AI14" s="19"/>
-    </row>
-    <row r="15" spans="1:35" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ14" s="19"/>
+      <c r="AK14" s="19"/>
+      <c r="AL14" s="19"/>
+    </row>
+    <row r="15" spans="1:38" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>33</v>
       </c>
@@ -2111,17 +2185,22 @@
         <v>214</v>
       </c>
       <c r="AD15" s="56" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="AE15" s="33"/>
       <c r="AF15" s="33"/>
       <c r="AG15" s="43" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="AH15" s="19"/>
       <c r="AI15" s="19"/>
-    </row>
-    <row r="16" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ15" s="43" t="s">
+        <v>247</v>
+      </c>
+      <c r="AK15" s="19"/>
+      <c r="AL15" s="19"/>
+    </row>
+    <row r="16" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
         <v>34</v>
       </c>
@@ -2141,8 +2220,11 @@
       <c r="AG16" s="19"/>
       <c r="AH16" s="19"/>
       <c r="AI16" s="19"/>
-    </row>
-    <row r="17" spans="1:35" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ16" s="19"/>
+      <c r="AK16" s="19"/>
+      <c r="AL16" s="19"/>
+    </row>
+    <row r="17" spans="1:38" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
         <v>35</v>
       </c>
@@ -2183,10 +2265,17 @@
       </c>
       <c r="AH17" s="19"/>
       <c r="AI17" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="18" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ17" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK17" s="19"/>
+      <c r="AL17" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>36</v>
       </c>
@@ -2206,8 +2295,11 @@
       <c r="AG18" s="19"/>
       <c r="AH18" s="19"/>
       <c r="AI18" s="19"/>
-    </row>
-    <row r="19" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ18" s="19"/>
+      <c r="AK18" s="19"/>
+      <c r="AL18" s="19"/>
+    </row>
+    <row r="19" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
         <v>37</v>
       </c>
@@ -2227,8 +2319,11 @@
       <c r="AG19" s="19"/>
       <c r="AH19" s="19"/>
       <c r="AI19" s="19"/>
-    </row>
-    <row r="20" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ19" s="19"/>
+      <c r="AK19" s="19"/>
+      <c r="AL19" s="19"/>
+    </row>
+    <row r="20" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>38</v>
       </c>
@@ -2254,8 +2349,11 @@
       <c r="AG20" s="19"/>
       <c r="AH20" s="19"/>
       <c r="AI20" s="19"/>
-    </row>
-    <row r="21" spans="1:35" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ20" s="19"/>
+      <c r="AK20" s="19"/>
+      <c r="AL20" s="19"/>
+    </row>
+    <row r="21" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A21" s="30" t="s">
         <v>39</v>
       </c>
@@ -2306,10 +2404,19 @@
         <v>206</v>
       </c>
       <c r="AI21" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="22" spans="1:35" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ21" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK21" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="AL21" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" spans="1:38" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A22" s="13" t="s">
         <v>40</v>
       </c>
@@ -2329,8 +2436,11 @@
       <c r="AG22" s="19"/>
       <c r="AH22" s="19"/>
       <c r="AI22" s="19"/>
-    </row>
-    <row r="23" spans="1:35" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ22" s="19"/>
+      <c r="AK22" s="19"/>
+      <c r="AL22" s="19"/>
+    </row>
+    <row r="23" spans="1:38" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A23" s="30" t="s">
         <v>41</v>
       </c>
@@ -2370,11 +2480,18 @@
         <v>166</v>
       </c>
       <c r="AH23" s="19" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="AI23" s="19"/>
-    </row>
-    <row r="24" spans="1:35" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="AJ23" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK23" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="AL23" s="19"/>
+    </row>
+    <row r="24" spans="1:38" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A24" s="19" t="s">
         <v>42</v>
       </c>
@@ -2394,8 +2511,11 @@
       <c r="AG24" s="19"/>
       <c r="AH24" s="19"/>
       <c r="AI24" s="19"/>
-    </row>
-    <row r="25" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ24" s="19"/>
+      <c r="AK24" s="19"/>
+      <c r="AL24" s="19"/>
+    </row>
+    <row r="25" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A25" s="30" t="s">
         <v>44</v>
       </c>
@@ -2448,8 +2568,11 @@
       <c r="AG25" s="19"/>
       <c r="AH25" s="19"/>
       <c r="AI25" s="19"/>
-    </row>
-    <row r="26" spans="1:35" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="AJ25" s="19"/>
+      <c r="AK25" s="19"/>
+      <c r="AL25" s="19"/>
+    </row>
+    <row r="26" spans="1:38" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
         <v>175</v>
       </c>
@@ -2477,10 +2600,17 @@
       </c>
       <c r="AH26" s="19"/>
       <c r="AI26" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="27" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ26" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK26" s="19"/>
+      <c r="AL26" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="27" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A27" s="30" t="s">
         <v>45</v>
       </c>
@@ -2516,8 +2646,11 @@
       <c r="AG27" s="19"/>
       <c r="AH27" s="19"/>
       <c r="AI27" s="19"/>
-    </row>
-    <row r="28" spans="1:35" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="AJ27" s="19"/>
+      <c r="AK27" s="19"/>
+      <c r="AL27" s="19"/>
+    </row>
+    <row r="28" spans="1:38" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
         <v>173</v>
       </c>
@@ -2545,10 +2678,17 @@
       </c>
       <c r="AH28" s="19"/>
       <c r="AI28" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="29" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ28" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK28" s="19"/>
+      <c r="AL28" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="29" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A29" s="30" t="s">
         <v>46</v>
       </c>
@@ -2584,10 +2724,17 @@
       </c>
       <c r="AH29" s="19"/>
       <c r="AI29" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="30" spans="1:35" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ29" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK29" s="19"/>
+      <c r="AL29" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="30" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A30" s="30" t="s">
         <v>47</v>
       </c>
@@ -2629,7 +2776,7 @@
         <v>207</v>
       </c>
       <c r="AD30" s="58" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="AE30" s="33"/>
       <c r="AF30" s="33"/>
@@ -2638,10 +2785,17 @@
       </c>
       <c r="AH30" s="19"/>
       <c r="AI30" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="31" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ30" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK30" s="19"/>
+      <c r="AL30" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="31" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A31" s="13" t="s">
         <v>48</v>
       </c>
@@ -2669,10 +2823,17 @@
       </c>
       <c r="AH31" s="19"/>
       <c r="AI31" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="32" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ31" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK31" s="19"/>
+      <c r="AL31" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="32" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A32" s="19" t="s">
         <v>49</v>
       </c>
@@ -2689,8 +2850,11 @@
       <c r="AG32" s="19"/>
       <c r="AH32" s="19"/>
       <c r="AI32" s="19"/>
-    </row>
-    <row r="33" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ32" s="19"/>
+      <c r="AK32" s="19"/>
+      <c r="AL32" s="19"/>
+    </row>
+    <row r="33" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A33" s="50">
         <v>2</v>
       </c>
@@ -2709,8 +2873,11 @@
       <c r="AG33" s="19"/>
       <c r="AH33" s="19"/>
       <c r="AI33" s="19"/>
-    </row>
-    <row r="34" spans="1:35" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ33" s="19"/>
+      <c r="AK33" s="19"/>
+      <c r="AL33" s="19"/>
+    </row>
+    <row r="34" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A34" s="30" t="s">
         <v>52</v>
       </c>
@@ -2735,8 +2902,11 @@
       <c r="AG34" s="19"/>
       <c r="AH34" s="19"/>
       <c r="AI34" s="19"/>
-    </row>
-    <row r="35" spans="1:35" ht="86.4" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ34" s="19"/>
+      <c r="AK34" s="19"/>
+      <c r="AL34" s="19"/>
+    </row>
+    <row r="35" spans="1:38" ht="409.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A35" s="13" t="s">
         <v>177</v>
       </c>
@@ -2781,26 +2951,35 @@
         <v>185</v>
       </c>
       <c r="AC35" s="19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AD35" s="60" t="s">
         <v>208</v>
       </c>
       <c r="AE35" s="33" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AF35" s="33" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="AG35" s="45" t="s">
         <v>167</v>
       </c>
       <c r="AH35" s="19"/>
       <c r="AI35" s="19" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="36" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+      <c r="AJ35" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK35" s="19" t="s">
+        <v>267</v>
+      </c>
+      <c r="AL35" s="19" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="36" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A36" s="13" t="s">
         <v>54</v>
       </c>
@@ -2841,8 +3020,11 @@
       <c r="AG36" s="19"/>
       <c r="AH36" s="19"/>
       <c r="AI36" s="19"/>
-    </row>
-    <row r="37" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ36" s="19"/>
+      <c r="AK36" s="19"/>
+      <c r="AL36" s="19"/>
+    </row>
+    <row r="37" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A37" s="13" t="s">
         <v>55</v>
       </c>
@@ -2871,8 +3053,11 @@
       <c r="AG37" s="19"/>
       <c r="AH37" s="19"/>
       <c r="AI37" s="19"/>
-    </row>
-    <row r="38" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ37" s="19"/>
+      <c r="AK37" s="19"/>
+      <c r="AL37" s="19"/>
+    </row>
+    <row r="38" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A38" s="13" t="s">
         <v>56</v>
       </c>
@@ -2895,8 +3080,11 @@
       <c r="AG38" s="19"/>
       <c r="AH38" s="19"/>
       <c r="AI38" s="19"/>
-    </row>
-    <row r="39" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ38" s="19"/>
+      <c r="AK38" s="19"/>
+      <c r="AL38" s="19"/>
+    </row>
+    <row r="39" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
         <v>57</v>
       </c>
@@ -2925,8 +3113,11 @@
       <c r="AG39" s="19"/>
       <c r="AH39" s="19"/>
       <c r="AI39" s="19"/>
-    </row>
-    <row r="40" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ39" s="19"/>
+      <c r="AK39" s="19"/>
+      <c r="AL39" s="19"/>
+    </row>
+    <row r="40" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
         <v>58</v>
       </c>
@@ -2955,8 +3146,11 @@
       <c r="AG40" s="19"/>
       <c r="AH40" s="19"/>
       <c r="AI40" s="19"/>
-    </row>
-    <row r="41" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ40" s="19"/>
+      <c r="AK40" s="19"/>
+      <c r="AL40" s="19"/>
+    </row>
+    <row r="41" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
         <v>59</v>
       </c>
@@ -2985,8 +3179,11 @@
       <c r="AG41" s="19"/>
       <c r="AH41" s="19"/>
       <c r="AI41" s="19"/>
-    </row>
-    <row r="42" spans="1:35" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="AJ41" s="19"/>
+      <c r="AK41" s="19"/>
+      <c r="AL41" s="19"/>
+    </row>
+    <row r="42" spans="1:38" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A42" s="13" t="s">
         <v>60</v>
       </c>
@@ -3015,8 +3212,11 @@
       <c r="AG42" s="19"/>
       <c r="AH42" s="19"/>
       <c r="AI42" s="19"/>
-    </row>
-    <row r="43" spans="1:35" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ42" s="19"/>
+      <c r="AK42" s="19"/>
+      <c r="AL42" s="19"/>
+    </row>
+    <row r="43" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A43" s="32" t="s">
         <v>62</v>
       </c>
@@ -3053,25 +3253,30 @@
         <v>220</v>
       </c>
       <c r="AB43" s="54" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AC43" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AD43" s="58" t="s">
         <v>220</v>
       </c>
       <c r="AE43" s="33"/>
       <c r="AF43" s="33" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AG43" s="47"/>
       <c r="AH43" s="19"/>
       <c r="AI43" s="19" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="44" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>221</v>
+      </c>
+      <c r="AJ43" s="47"/>
+      <c r="AK43" s="19"/>
+      <c r="AL43" s="19" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="44" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C44" s="25" t="s">
         <v>63</v>
       </c>
@@ -3103,10 +3308,13 @@
       <c r="AG44" s="47"/>
       <c r="AH44" s="19"/>
       <c r="AI44" s="19"/>
-    </row>
-    <row r="45" spans="1:35" ht="72" x14ac:dyDescent="0.3">
+      <c r="AJ44" s="47"/>
+      <c r="AK44" s="19"/>
+      <c r="AL44" s="19"/>
+    </row>
+    <row r="45" spans="1:38" ht="72" x14ac:dyDescent="0.3">
       <c r="A45" s="50" t="s">
-        <v>221</v>
+        <v>269</v>
       </c>
       <c r="B45" s="16" t="s">
         <v>64</v>
@@ -3136,7 +3344,7 @@
         <v>219</v>
       </c>
       <c r="AC45" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AD45" s="58" t="s">
         <v>209</v>
@@ -3145,19 +3353,28 @@
         <v>219</v>
       </c>
       <c r="AF45" s="33" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AG45" s="44" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="AH45" s="19" t="s">
         <v>219</v>
       </c>
       <c r="AI45" s="19" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="46" spans="1:35" ht="28.8" outlineLevel="2" x14ac:dyDescent="0.3">
+        <v>263</v>
+      </c>
+      <c r="AJ45" s="44" t="s">
+        <v>262</v>
+      </c>
+      <c r="AK45" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="AL45" s="19" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="46" spans="1:38" ht="28.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A46" s="19" t="s">
         <v>66</v>
       </c>
@@ -3210,8 +3427,15 @@
         <v>210</v>
       </c>
       <c r="AI46" s="19"/>
-    </row>
-    <row r="47" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ46" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK46" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="AL46" s="19"/>
+    </row>
+    <row r="47" spans="1:38" ht="43.2" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A47" s="19" t="s">
         <v>67</v>
       </c>
@@ -3264,8 +3488,15 @@
         <v>210</v>
       </c>
       <c r="AI47" s="19"/>
-    </row>
-    <row r="48" spans="1:35" ht="86.4" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ47" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK47" s="63" t="s">
+        <v>268</v>
+      </c>
+      <c r="AL47" s="19"/>
+    </row>
+    <row r="48" spans="1:38" ht="86.4" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A48" s="33" t="s">
         <v>68</v>
       </c>
@@ -3321,10 +3552,17 @@
         <v>186</v>
       </c>
       <c r="AI48" s="19"/>
-    </row>
-    <row r="49" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ48" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK48" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="AL48" s="19"/>
+    </row>
+    <row r="49" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A49" s="32" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D49" s="33"/>
       <c r="E49" s="6"/>
@@ -3339,10 +3577,15 @@
       </c>
       <c r="AH49" s="19"/>
       <c r="AI49" s="19"/>
-    </row>
-    <row r="50" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ49" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK49" s="19"/>
+      <c r="AL49" s="19"/>
+    </row>
+    <row r="50" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A50" s="32" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D50" s="33"/>
       <c r="E50" s="6"/>
@@ -3360,10 +3603,15 @@
       </c>
       <c r="AH50" s="19"/>
       <c r="AI50" s="19"/>
-    </row>
-    <row r="51" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ50" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK50" s="19"/>
+      <c r="AL50" s="19"/>
+    </row>
+    <row r="51" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A51" s="32" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D51" s="33"/>
       <c r="E51" s="6"/>
@@ -3381,10 +3629,15 @@
       </c>
       <c r="AH51" s="19"/>
       <c r="AI51" s="19"/>
-    </row>
-    <row r="52" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ51" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK51" s="19"/>
+      <c r="AL51" s="19"/>
+    </row>
+    <row r="52" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A52" s="32" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D52" s="33"/>
       <c r="E52" s="6"/>
@@ -3402,10 +3655,15 @@
       </c>
       <c r="AH52" s="19"/>
       <c r="AI52" s="19"/>
-    </row>
-    <row r="53" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ52" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK52" s="19"/>
+      <c r="AL52" s="19"/>
+    </row>
+    <row r="53" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A53" s="32" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D53" s="33"/>
       <c r="E53" s="6"/>
@@ -3423,10 +3681,15 @@
       </c>
       <c r="AH53" s="19"/>
       <c r="AI53" s="19"/>
-    </row>
-    <row r="54" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ53" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK53" s="19"/>
+      <c r="AL53" s="19"/>
+    </row>
+    <row r="54" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A54" s="32" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D54" s="33"/>
       <c r="E54" s="6"/>
@@ -3444,10 +3707,15 @@
       </c>
       <c r="AH54" s="19"/>
       <c r="AI54" s="19"/>
-    </row>
-    <row r="55" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ54" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK54" s="19"/>
+      <c r="AL54" s="19"/>
+    </row>
+    <row r="55" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A55" s="32" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D55" s="33"/>
       <c r="E55" s="6"/>
@@ -3465,10 +3733,15 @@
       </c>
       <c r="AH55" s="19"/>
       <c r="AI55" s="19"/>
-    </row>
-    <row r="56" spans="1:35" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ55" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK55" s="19"/>
+      <c r="AL55" s="19"/>
+    </row>
+    <row r="56" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A56" s="32" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D56" s="33"/>
       <c r="E56" s="6"/>
@@ -3486,8 +3759,13 @@
       </c>
       <c r="AH56" s="19"/>
       <c r="AI56" s="19"/>
-    </row>
-    <row r="57" spans="1:35" ht="72" outlineLevel="2" x14ac:dyDescent="0.3">
+      <c r="AJ56" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="AK56" s="19"/>
+      <c r="AL56" s="19"/>
+    </row>
+    <row r="57" spans="1:38" ht="72" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A57" s="33" t="s">
         <v>171</v>
       </c>
@@ -3530,20 +3808,27 @@
         <v>167</v>
       </c>
       <c r="AE57" s="62" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="AF57" s="33"/>
       <c r="AG57" s="45" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="AH57" s="55" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="AI57" s="19"/>
-    </row>
-    <row r="58" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ57" s="45" t="s">
+        <v>246</v>
+      </c>
+      <c r="AK57" s="55" t="s">
+        <v>241</v>
+      </c>
+      <c r="AL57" s="19"/>
+    </row>
+    <row r="58" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A58" s="50" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B58" s="16" t="s">
         <v>69</v>
@@ -3576,13 +3861,16 @@
       <c r="AG58" s="19"/>
       <c r="AH58" s="19"/>
       <c r="AI58" s="19"/>
-    </row>
-    <row r="59" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ58" s="19"/>
+      <c r="AK58" s="19"/>
+      <c r="AL58" s="19"/>
+    </row>
+    <row r="59" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A59" s="32" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D59" s="32" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E59" s="6"/>
       <c r="F59" s="6"/>
@@ -3601,13 +3889,18 @@
       </c>
       <c r="AH59" s="19"/>
       <c r="AI59" s="19"/>
-    </row>
-    <row r="60" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ59" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK59" s="19"/>
+      <c r="AL59" s="19"/>
+    </row>
+    <row r="60" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A60" s="32" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D60" s="32" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E60" s="6"/>
       <c r="F60" s="6"/>
@@ -3625,13 +3918,18 @@
       </c>
       <c r="AH60" s="19"/>
       <c r="AI60" s="19"/>
-    </row>
-    <row r="61" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ60" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK60" s="19"/>
+      <c r="AL60" s="19"/>
+    </row>
+    <row r="61" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A61" s="32" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D61" s="32" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E61" s="6"/>
       <c r="F61" s="6"/>
@@ -3649,13 +3947,18 @@
       </c>
       <c r="AH61" s="19"/>
       <c r="AI61" s="19"/>
-    </row>
-    <row r="62" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ61" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK61" s="19"/>
+      <c r="AL61" s="19"/>
+    </row>
+    <row r="62" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A62" s="32" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D62" s="32" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E62" s="6"/>
       <c r="F62" s="6"/>
@@ -3671,13 +3974,16 @@
       <c r="AG62" s="19"/>
       <c r="AH62" s="19"/>
       <c r="AI62" s="19"/>
-    </row>
-    <row r="63" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ62" s="19"/>
+      <c r="AK62" s="19"/>
+      <c r="AL62" s="19"/>
+    </row>
+    <row r="63" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A63" s="32" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D63" s="32" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="E63" s="6"/>
       <c r="F63" s="6"/>
@@ -3695,13 +4001,18 @@
       </c>
       <c r="AH63" s="19"/>
       <c r="AI63" s="19"/>
-    </row>
-    <row r="64" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ63" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK63" s="19"/>
+      <c r="AL63" s="19"/>
+    </row>
+    <row r="64" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A64" s="32" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D64" s="32" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
@@ -3719,13 +4030,18 @@
       </c>
       <c r="AH64" s="19"/>
       <c r="AI64" s="19"/>
-    </row>
-    <row r="65" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ64" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK64" s="19"/>
+      <c r="AL64" s="19"/>
+    </row>
+    <row r="65" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A65" s="32" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D65" s="32" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
@@ -3743,13 +4059,18 @@
       </c>
       <c r="AH65" s="19"/>
       <c r="AI65" s="19"/>
-    </row>
-    <row r="66" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ65" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK65" s="19"/>
+      <c r="AL65" s="19"/>
+    </row>
+    <row r="66" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A66" s="32" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D66" s="32" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
@@ -3765,8 +4086,11 @@
       <c r="AG66" s="19"/>
       <c r="AH66" s="19"/>
       <c r="AI66" s="19"/>
-    </row>
-    <row r="67" spans="1:35" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ66" s="19"/>
+      <c r="AK66" s="19"/>
+      <c r="AL66" s="19"/>
+    </row>
+    <row r="67" spans="1:38" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A67" s="30" t="s">
         <v>71</v>
       </c>
@@ -3806,14 +4130,21 @@
       </c>
       <c r="AF67" s="33"/>
       <c r="AG67" s="46" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AH67" s="19" t="s">
         <v>187</v>
       </c>
       <c r="AI67" s="19"/>
-    </row>
-    <row r="68" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ67" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="AK67" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="AL67" s="19"/>
+    </row>
+    <row r="68" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D68" s="13" t="s">
         <v>72</v>
       </c>
@@ -3821,8 +4152,11 @@
       <c r="AG68" s="19"/>
       <c r="AH68" s="19"/>
       <c r="AI68" s="19"/>
-    </row>
-    <row r="69" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ68" s="19"/>
+      <c r="AK68" s="19"/>
+      <c r="AL68" s="19"/>
+    </row>
+    <row r="69" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D69" s="13" t="s">
         <v>73</v>
       </c>
@@ -3830,8 +4164,11 @@
       <c r="AG69" s="19"/>
       <c r="AH69" s="19"/>
       <c r="AI69" s="19"/>
-    </row>
-    <row r="70" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ69" s="19"/>
+      <c r="AK69" s="19"/>
+      <c r="AL69" s="19"/>
+    </row>
+    <row r="70" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D70" s="13" t="s">
         <v>74</v>
       </c>
@@ -3839,8 +4176,11 @@
       <c r="AG70" s="19"/>
       <c r="AH70" s="19"/>
       <c r="AI70" s="19"/>
-    </row>
-    <row r="71" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ70" s="19"/>
+      <c r="AK70" s="19"/>
+      <c r="AL70" s="19"/>
+    </row>
+    <row r="71" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D71" s="13" t="s">
         <v>75</v>
       </c>
@@ -3848,8 +4188,11 @@
       <c r="AG71" s="19"/>
       <c r="AH71" s="19"/>
       <c r="AI71" s="19"/>
-    </row>
-    <row r="72" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ71" s="19"/>
+      <c r="AK71" s="19"/>
+      <c r="AL71" s="19"/>
+    </row>
+    <row r="72" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D72" s="13" t="s">
         <v>76</v>
       </c>
@@ -3857,8 +4200,11 @@
       <c r="AG72" s="19"/>
       <c r="AH72" s="19"/>
       <c r="AI72" s="19"/>
-    </row>
-    <row r="73" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ72" s="19"/>
+      <c r="AK72" s="19"/>
+      <c r="AL72" s="19"/>
+    </row>
+    <row r="73" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D73" s="13" t="s">
         <v>77</v>
       </c>
@@ -3866,8 +4212,11 @@
       <c r="AG73" s="19"/>
       <c r="AH73" s="19"/>
       <c r="AI73" s="19"/>
-    </row>
-    <row r="74" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ73" s="19"/>
+      <c r="AK73" s="19"/>
+      <c r="AL73" s="19"/>
+    </row>
+    <row r="74" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D74" s="13" t="s">
         <v>78</v>
       </c>
@@ -3887,8 +4236,11 @@
       <c r="AG74" s="19"/>
       <c r="AH74" s="19"/>
       <c r="AI74" s="19"/>
-    </row>
-    <row r="75" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ74" s="19"/>
+      <c r="AK74" s="19"/>
+      <c r="AL74" s="19"/>
+    </row>
+    <row r="75" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D75" s="13" t="s">
         <v>79</v>
       </c>
@@ -3908,8 +4260,11 @@
       <c r="AG75" s="19"/>
       <c r="AH75" s="19"/>
       <c r="AI75" s="19"/>
-    </row>
-    <row r="76" spans="1:35" ht="115.2" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="AJ75" s="19"/>
+      <c r="AK75" s="19"/>
+      <c r="AL75" s="19"/>
+    </row>
+    <row r="76" spans="1:38" ht="115.2" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
       <c r="A76" s="23" t="s">
         <v>80</v>
       </c>
@@ -3960,13 +4315,22 @@
         <v>165</v>
       </c>
       <c r="AH76" s="55" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="AI76" s="19" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="77" spans="1:35" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ76" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK76" s="55" t="s">
+        <v>238</v>
+      </c>
+      <c r="AL76" s="19" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="77" spans="1:38" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A77" s="13" t="s">
         <v>82</v>
       </c>
@@ -3998,17 +4362,24 @@
         <v>165</v>
       </c>
       <c r="AB77" s="55" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AG77" s="43" t="s">
         <v>165</v>
       </c>
       <c r="AH77" s="55" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AI77" s="19"/>
-    </row>
-    <row r="78" spans="1:35" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ77" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK77" s="55" t="s">
+        <v>235</v>
+      </c>
+      <c r="AL77" s="19"/>
+    </row>
+    <row r="78" spans="1:38" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A78" s="13" t="s">
         <v>191</v>
       </c>
@@ -4055,16 +4426,25 @@
         <v>188</v>
       </c>
       <c r="AG78" s="43" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="AH78" s="55" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="AI78" s="19" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="79" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ78" s="43" t="s">
+        <v>234</v>
+      </c>
+      <c r="AK78" s="55" t="s">
+        <v>239</v>
+      </c>
+      <c r="AL78" s="19" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="79" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A79" s="13" t="s">
         <v>83</v>
       </c>
@@ -4103,8 +4483,13 @@
       </c>
       <c r="AH79" s="19"/>
       <c r="AI79" s="19"/>
-    </row>
-    <row r="80" spans="1:35" ht="72" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ79" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK79" s="19"/>
+      <c r="AL79" s="19"/>
+    </row>
+    <row r="80" spans="1:38" ht="72" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A80" s="13" t="s">
         <v>84</v>
       </c>
@@ -4139,20 +4524,27 @@
         <v>192</v>
       </c>
       <c r="AA80" s="44" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AB80" s="19" t="s">
         <v>213</v>
       </c>
       <c r="AG80" s="44" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AH80" s="19" t="s">
         <v>213</v>
       </c>
       <c r="AI80" s="19"/>
-    </row>
-    <row r="81" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ80" s="44" t="s">
+        <v>236</v>
+      </c>
+      <c r="AK80" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="AL80" s="19"/>
+    </row>
+    <row r="81" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A81" s="13" t="s">
         <v>85</v>
       </c>
@@ -4177,8 +4569,11 @@
       <c r="AG81" s="19"/>
       <c r="AH81" s="19"/>
       <c r="AI81" s="19"/>
-    </row>
-    <row r="82" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ81" s="19"/>
+      <c r="AK81" s="19"/>
+      <c r="AL81" s="19"/>
+    </row>
+    <row r="82" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A82" s="13" t="s">
         <v>79</v>
       </c>
@@ -4207,8 +4602,11 @@
       <c r="AG82" s="19"/>
       <c r="AH82" s="19"/>
       <c r="AI82" s="19"/>
-    </row>
-    <row r="83" spans="1:35" ht="72" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ82" s="19"/>
+      <c r="AK82" s="19"/>
+      <c r="AL82" s="19"/>
+    </row>
+    <row r="83" spans="1:38" ht="72" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A83" s="13" t="s">
         <v>86</v>
       </c>
@@ -4249,8 +4647,17 @@
       <c r="AI83" s="19" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="84" spans="1:35" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ83" s="46" t="s">
+        <v>170</v>
+      </c>
+      <c r="AK83" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="AL83" s="19" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="84" spans="1:38" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A84" s="13" t="s">
         <v>87</v>
       </c>
@@ -4294,8 +4701,17 @@
       <c r="AI84" s="19" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="85" spans="1:35" ht="72" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ84" s="46" t="s">
+        <v>172</v>
+      </c>
+      <c r="AK84" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="AL84" s="19" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="85" spans="1:38" ht="100.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A85" s="13" t="s">
         <v>88</v>
       </c>
@@ -4331,7 +4747,7 @@
         <v>201</v>
       </c>
       <c r="AG85" s="46" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="AH85" s="19" t="s">
         <v>193</v>
@@ -4339,8 +4755,17 @@
       <c r="AI85" s="19" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="86" spans="1:35" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="AJ85" s="46" t="s">
+        <v>242</v>
+      </c>
+      <c r="AK85" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="AL85" s="19" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="86" spans="1:38" ht="23.4" x14ac:dyDescent="0.3">
       <c r="A86" s="50">
         <v>4</v>
       </c>
@@ -4356,8 +4781,11 @@
       <c r="AG86" s="19"/>
       <c r="AH86" s="19"/>
       <c r="AI86" s="19"/>
-    </row>
-    <row r="87" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ86" s="19"/>
+      <c r="AK86" s="19"/>
+      <c r="AL86" s="19"/>
+    </row>
+    <row r="87" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A87" s="49" t="s">
         <v>216</v>
       </c>
@@ -4400,8 +4828,13 @@
       </c>
       <c r="AH87" s="19"/>
       <c r="AI87" s="19"/>
-    </row>
-    <row r="88" spans="1:35" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ87" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK87" s="19"/>
+      <c r="AL87" s="19"/>
+    </row>
+    <row r="88" spans="1:38" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A88" s="49" t="s">
         <v>217</v>
       </c>
@@ -4446,22 +4879,31 @@
         <v>168</v>
       </c>
       <c r="AB88" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AC88" s="19" t="s">
         <v>196</v>
       </c>
       <c r="AG88" s="43" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="AH88" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AI88" s="19" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="89" spans="1:35" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>265</v>
+      </c>
+      <c r="AJ88" s="43" t="s">
+        <v>266</v>
+      </c>
+      <c r="AK88" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="AL88" s="19" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="89" spans="1:38" ht="100.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A89" s="30" t="s">
         <v>95</v>
       </c>
@@ -4505,17 +4947,24 @@
         <v>168</v>
       </c>
       <c r="AB89" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AG89" s="45" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="AH89" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AI89" s="19"/>
-    </row>
-    <row r="90" spans="1:35" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ89" s="45" t="s">
+        <v>237</v>
+      </c>
+      <c r="AK89" s="19" t="s">
+        <v>230</v>
+      </c>
+      <c r="AL89" s="19"/>
+    </row>
+    <row r="90" spans="1:38" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A90" s="30" t="s">
         <v>97</v>
       </c>
@@ -4547,17 +4996,22 @@
         <v>168</v>
       </c>
       <c r="AB90" s="19" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AG90" s="19"/>
       <c r="AH90" s="19" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AI90" s="19"/>
-    </row>
-    <row r="91" spans="1:35" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ90" s="19"/>
+      <c r="AK90" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="AL90" s="19"/>
+    </row>
+    <row r="91" spans="1:38" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A91" s="30" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B91" s="15"/>
       <c r="C91" s="23" t="s">
@@ -4586,19 +5040,26 @@
         <v>166</v>
       </c>
       <c r="AC91" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AG91" s="44" t="s">
         <v>166</v>
       </c>
       <c r="AH91" s="19"/>
       <c r="AI91" s="19" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="92" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>227</v>
+      </c>
+      <c r="AJ91" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK91" s="19"/>
+      <c r="AL91" s="19" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="92" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A92" s="30" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B92" s="15"/>
       <c r="C92" s="23"/>
@@ -4623,8 +5084,13 @@
       </c>
       <c r="AH92" s="19"/>
       <c r="AI92" s="19"/>
-    </row>
-    <row r="93" spans="1:35" ht="86.4" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ92" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK92" s="19"/>
+      <c r="AL92" s="19"/>
+    </row>
+    <row r="93" spans="1:38" ht="86.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A93" s="30" t="s">
         <v>100</v>
       </c>
@@ -4658,17 +5124,24 @@
         <v>168</v>
       </c>
       <c r="AB93" s="19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AG93" s="45" t="s">
         <v>167</v>
       </c>
       <c r="AH93" s="19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AI93" s="19"/>
-    </row>
-    <row r="94" spans="1:35" ht="63" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ93" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK93" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="AL93" s="19"/>
+    </row>
+    <row r="94" spans="1:38" ht="63" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A94" s="30" t="s">
         <v>102</v>
       </c>
@@ -4717,8 +5190,15 @@
       <c r="AI94" s="19" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="95" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ94" s="19"/>
+      <c r="AK94" s="53">
+        <v>46309</v>
+      </c>
+      <c r="AL94" s="19" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="95" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A95" s="13" t="s">
         <v>104</v>
       </c>
@@ -4746,8 +5226,13 @@
       </c>
       <c r="AH95" s="19"/>
       <c r="AI95" s="19"/>
-    </row>
-    <row r="96" spans="1:35" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ95" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="AK95" s="19"/>
+      <c r="AL95" s="19"/>
+    </row>
+    <row r="96" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A96" s="30" t="s">
         <v>105</v>
       </c>
@@ -4797,8 +5282,17 @@
       <c r="AI96" s="19" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="97" spans="1:35" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ96" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="AK96" s="53">
+        <v>46314</v>
+      </c>
+      <c r="AL96" s="19" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="97" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A97" s="30" t="s">
         <v>107</v>
       </c>
@@ -4847,8 +5341,17 @@
       <c r="AI97" s="19" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="98" spans="1:35" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ97" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="AK97" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="AL97" s="19" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="98" spans="1:38" ht="86.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>109</v>
       </c>
@@ -4884,25 +5387,32 @@
         <v>168</v>
       </c>
       <c r="AB98" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="AC98" s="19" t="s">
         <v>226</v>
       </c>
-      <c r="AC98" s="19" t="s">
-        <v>227</v>
-      </c>
       <c r="AG98" s="43" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="AH98" s="19"/>
       <c r="AI98" s="19" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="99" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+      <c r="AJ98" s="43" t="s">
+        <v>245</v>
+      </c>
+      <c r="AK98" s="19"/>
+      <c r="AL98" s="19" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="99" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
-        <v>249</v>
+        <v>270</v>
       </c>
       <c r="C99" s="16" t="s">
-        <v>248</v>
+        <v>272</v>
       </c>
       <c r="D99" s="13"/>
       <c r="E99" s="6"/>
@@ -4919,75 +5429,76 @@
       <c r="AG99" s="43"/>
       <c r="AH99" s="19"/>
       <c r="AI99" s="19"/>
-    </row>
-    <row r="100" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A100" s="50" t="s">
-        <v>224</v>
-      </c>
-      <c r="B100" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="C100" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="M100" s="28">
-        <v>156</v>
-      </c>
-      <c r="X100" s="37" t="s">
-        <v>203</v>
-      </c>
-      <c r="AA100" s="46" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG100" s="46" t="s">
-        <v>203</v>
-      </c>
+      <c r="AJ99" s="43"/>
+      <c r="AK99" s="19"/>
+      <c r="AL99" s="19"/>
+    </row>
+    <row r="100" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="C100" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="D100" s="13"/>
+      <c r="E100" s="6"/>
+      <c r="F100" s="6"/>
+      <c r="G100" s="6"/>
+      <c r="H100" s="11"/>
+      <c r="I100" s="6"/>
+      <c r="J100" s="6"/>
+      <c r="K100" s="6"/>
+      <c r="L100" s="6"/>
+      <c r="M100" s="26"/>
+      <c r="X100" s="37"/>
+      <c r="AA100" s="46"/>
+      <c r="AG100" s="43"/>
       <c r="AH100" s="19"/>
       <c r="AI100" s="19"/>
-    </row>
-    <row r="101" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B101" s="18"/>
-      <c r="C101" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="D101" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="E101" s="6"/>
-      <c r="F101" s="6"/>
-      <c r="G101" s="6"/>
-      <c r="H101" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="J101" s="6"/>
-      <c r="K101" s="6"/>
-      <c r="L101" s="6"/>
-      <c r="M101" s="26"/>
+      <c r="AJ100" s="43"/>
+      <c r="AK100" s="19"/>
+      <c r="AL100" s="19"/>
+    </row>
+    <row r="101" spans="1:38" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A101" s="50" t="s">
+        <v>223</v>
+      </c>
+      <c r="B101" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C101" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="M101" s="28">
+        <v>156</v>
+      </c>
       <c r="X101" s="37" t="s">
-        <v>168</v>
+        <v>203</v>
       </c>
       <c r="AA101" s="46" t="s">
-        <v>168</v>
+        <v>203</v>
       </c>
       <c r="AG101" s="46" t="s">
-        <v>168</v>
+        <v>203</v>
       </c>
       <c r="AH101" s="19"/>
       <c r="AI101" s="19"/>
-    </row>
-    <row r="102" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ101" s="46" t="s">
+        <v>203</v>
+      </c>
+      <c r="AK101" s="19"/>
+      <c r="AL101" s="19"/>
+    </row>
+    <row r="102" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B102" s="18"/>
       <c r="C102" s="16" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E102" s="6"/>
       <c r="F102" s="6"/>
@@ -5010,32 +5521,56 @@
       </c>
       <c r="AH102" s="19"/>
       <c r="AI102" s="19"/>
-    </row>
-    <row r="103" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A103"/>
+      <c r="AJ102" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="AK102" s="19"/>
+      <c r="AL102" s="19"/>
+    </row>
+    <row r="103" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="B103" s="18"/>
-      <c r="C103"/>
+      <c r="C103" s="16" t="s">
+        <v>116</v>
+      </c>
       <c r="D103" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E103" s="6"/>
       <c r="F103" s="6"/>
       <c r="G103" s="6"/>
-      <c r="H103" s="21"/>
+      <c r="H103" s="21" t="s">
+        <v>115</v>
+      </c>
       <c r="J103" s="6"/>
       <c r="K103" s="6"/>
       <c r="L103" s="6"/>
       <c r="M103" s="26"/>
-      <c r="AG103" s="19"/>
+      <c r="X103" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="AA103" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="AG103" s="46" t="s">
+        <v>168</v>
+      </c>
       <c r="AH103" s="19"/>
       <c r="AI103" s="19"/>
-    </row>
-    <row r="104" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ103" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="AK103" s="19"/>
+      <c r="AL103" s="19"/>
+    </row>
+    <row r="104" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A104"/>
       <c r="B104" s="18"/>
       <c r="C104"/>
       <c r="D104" s="13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E104" s="6"/>
       <c r="F104" s="6"/>
@@ -5048,13 +5583,16 @@
       <c r="AG104" s="19"/>
       <c r="AH104" s="19"/>
       <c r="AI104" s="19"/>
-    </row>
-    <row r="105" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ104" s="19"/>
+      <c r="AK104" s="19"/>
+      <c r="AL104" s="19"/>
+    </row>
+    <row r="105" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A105"/>
       <c r="B105" s="18"/>
       <c r="C105"/>
       <c r="D105" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E105" s="6"/>
       <c r="F105" s="6"/>
@@ -5067,13 +5605,16 @@
       <c r="AG105" s="19"/>
       <c r="AH105" s="19"/>
       <c r="AI105" s="19"/>
-    </row>
-    <row r="106" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ105" s="19"/>
+      <c r="AK105" s="19"/>
+      <c r="AL105" s="19"/>
+    </row>
+    <row r="106" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A106"/>
       <c r="B106" s="18"/>
       <c r="C106"/>
       <c r="D106" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E106" s="6"/>
       <c r="F106" s="6"/>
@@ -5086,13 +5627,16 @@
       <c r="AG106" s="19"/>
       <c r="AH106" s="19"/>
       <c r="AI106" s="19"/>
-    </row>
-    <row r="107" spans="1:35" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="AJ106" s="19"/>
+      <c r="AK106" s="19"/>
+      <c r="AL106" s="19"/>
+    </row>
+    <row r="107" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A107"/>
       <c r="B107" s="18"/>
       <c r="C107"/>
       <c r="D107" s="13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E107" s="6"/>
       <c r="F107" s="6"/>
@@ -5105,85 +5649,104 @@
       <c r="AG107" s="19"/>
       <c r="AH107" s="19"/>
       <c r="AI107" s="19"/>
-    </row>
-    <row r="108" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="5" t="s">
-        <v>123</v>
-      </c>
+      <c r="AJ107" s="19"/>
+      <c r="AK107" s="19"/>
+      <c r="AL107" s="19"/>
+    </row>
+    <row r="108" spans="1:38" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.3">
+      <c r="A108"/>
       <c r="B108" s="18"/>
-      <c r="C108" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="D108" s="13"/>
+      <c r="C108"/>
+      <c r="D108" s="13" t="s">
+        <v>122</v>
+      </c>
       <c r="E108" s="6"/>
       <c r="F108" s="6"/>
       <c r="G108" s="6"/>
-      <c r="H108" s="21" t="s">
-        <v>115</v>
-      </c>
+      <c r="H108" s="21"/>
       <c r="J108" s="6"/>
       <c r="K108" s="6"/>
       <c r="L108" s="6"/>
       <c r="M108" s="26"/>
-      <c r="X108" s="42" t="s">
-        <v>202</v>
-      </c>
-      <c r="AA108" s="45" t="s">
-        <v>167</v>
-      </c>
-      <c r="AG108" s="45" t="s">
-        <v>167</v>
-      </c>
+      <c r="AG108" s="19"/>
       <c r="AH108" s="19"/>
       <c r="AI108" s="19"/>
-    </row>
-    <row r="109" spans="1:35" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A109" s="50" t="s">
-        <v>225</v>
-      </c>
-      <c r="B109" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="C109" s="24" t="s">
-        <v>125</v>
-      </c>
-      <c r="M109" s="28">
-        <v>89</v>
-      </c>
-      <c r="X109" s="37" t="s">
-        <v>203</v>
-      </c>
-      <c r="AA109" s="46" t="s">
-        <v>203</v>
-      </c>
-      <c r="AG109" s="46" t="s">
-        <v>203</v>
+      <c r="AJ108" s="19"/>
+      <c r="AK108" s="19"/>
+      <c r="AL108" s="19"/>
+    </row>
+    <row r="109" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B109" s="18"/>
+      <c r="C109" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="D109" s="13"/>
+      <c r="E109" s="6"/>
+      <c r="F109" s="6"/>
+      <c r="G109" s="6"/>
+      <c r="H109" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="J109" s="6"/>
+      <c r="K109" s="6"/>
+      <c r="L109" s="6"/>
+      <c r="M109" s="26"/>
+      <c r="X109" s="42" t="s">
+        <v>202</v>
+      </c>
+      <c r="AA109" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AG109" s="45" t="s">
+        <v>167</v>
       </c>
       <c r="AH109" s="19"/>
       <c r="AI109" s="19"/>
-    </row>
-    <row r="110" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="48"/>
-      <c r="B110" s="18"/>
-      <c r="C110" s="16"/>
-      <c r="D110" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E110" s="6"/>
-      <c r="F110" s="6"/>
-      <c r="G110" s="6"/>
-      <c r="H110" s="21"/>
-      <c r="J110" s="6"/>
-      <c r="K110" s="6"/>
-      <c r="L110" s="6"/>
-      <c r="M110" s="26"/>
-    </row>
-    <row r="111" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="AJ109" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="AK109" s="19"/>
+      <c r="AL109" s="19"/>
+    </row>
+    <row r="110" spans="1:38" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A110" s="50" t="s">
+        <v>224</v>
+      </c>
+      <c r="B110" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C110" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="M110" s="28">
+        <v>89</v>
+      </c>
+      <c r="X110" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="AA110" s="46" t="s">
+        <v>203</v>
+      </c>
+      <c r="AG110" s="46" t="s">
+        <v>203</v>
+      </c>
+      <c r="AH110" s="19"/>
+      <c r="AI110" s="19"/>
+      <c r="AJ110" s="46" t="s">
+        <v>203</v>
+      </c>
+      <c r="AK110" s="19"/>
+      <c r="AL110" s="19"/>
+    </row>
+    <row r="111" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A111" s="48"/>
       <c r="B111" s="18"/>
       <c r="C111" s="16"/>
       <c r="D111" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E111" s="6"/>
       <c r="F111" s="6"/>
@@ -5194,12 +5757,12 @@
       <c r="L111" s="6"/>
       <c r="M111" s="26"/>
     </row>
-    <row r="112" spans="1:35" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A112" s="48"/>
       <c r="B112" s="18"/>
       <c r="C112" s="16"/>
       <c r="D112" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E112" s="6"/>
       <c r="F112" s="6"/>
@@ -5215,7 +5778,7 @@
       <c r="B113" s="18"/>
       <c r="C113" s="16"/>
       <c r="D113" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E113" s="6"/>
       <c r="F113" s="6"/>
@@ -5226,36 +5789,38 @@
       <c r="L113" s="6"/>
       <c r="M113" s="26"/>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:13" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A114" s="48"/>
       <c r="B114" s="18"/>
-      <c r="C114" s="18"/>
-      <c r="D114" s="18"/>
-      <c r="E114" s="18"/>
-      <c r="F114" s="18"/>
-      <c r="G114" s="18"/>
-      <c r="H114" s="18"/>
-      <c r="I114" s="19"/>
-      <c r="J114" s="12"/>
-      <c r="K114" s="17"/>
-      <c r="L114" s="17"/>
-      <c r="M114" s="17"/>
+      <c r="C114" s="16"/>
+      <c r="D114" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="E114" s="6"/>
+      <c r="F114" s="6"/>
+      <c r="G114" s="6"/>
+      <c r="H114" s="21"/>
+      <c r="J114" s="6"/>
+      <c r="K114" s="6"/>
+      <c r="L114" s="6"/>
+      <c r="M114" s="26"/>
     </row>
     <row r="115" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D115" s="12"/>
-      <c r="E115" s="6"/>
-      <c r="F115" s="6"/>
-      <c r="G115" s="6"/>
-      <c r="H115" s="6"/>
-      <c r="I115" s="6"/>
-      <c r="J115" s="6"/>
+      <c r="A115" s="48"/>
+      <c r="B115" s="18"/>
+      <c r="C115" s="18"/>
+      <c r="D115" s="18"/>
+      <c r="E115" s="18"/>
+      <c r="F115" s="18"/>
+      <c r="G115" s="18"/>
+      <c r="H115" s="18"/>
+      <c r="I115" s="19"/>
+      <c r="J115" s="12"/>
       <c r="K115" s="17"/>
       <c r="L115" s="17"/>
       <c r="M115" s="17"/>
     </row>
-    <row r="116" spans="1:13" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="A116" s="51"/>
-      <c r="B116" s="8"/>
+    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
       <c r="D116" s="12"/>
       <c r="E116" s="6"/>
       <c r="F116" s="6"/>
@@ -5265,38 +5830,52 @@
       <c r="J116" s="6"/>
       <c r="K116" s="17"/>
       <c r="L116" s="17"/>
-      <c r="M116" s="29">
-        <f>M3+M10+M33+M45+M58+M86+M100+M109</f>
+      <c r="M116" s="17"/>
+    </row>
+    <row r="117" spans="1:13" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="A117" s="51"/>
+      <c r="B117" s="8"/>
+      <c r="D117" s="12"/>
+      <c r="E117" s="6"/>
+      <c r="F117" s="6"/>
+      <c r="G117" s="6"/>
+      <c r="H117" s="6"/>
+      <c r="I117" s="6"/>
+      <c r="J117" s="6"/>
+      <c r="K117" s="17"/>
+      <c r="L117" s="17"/>
+      <c r="M117" s="29">
+        <f>M3+M10+M33+M45+M58+M86+M101+M110</f>
         <v>825</v>
       </c>
     </row>
-    <row r="121" spans="1:13" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A121" s="52" t="s">
+    <row r="122" spans="1:13" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A122" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="B121" s="1"/>
-    </row>
-    <row r="122" spans="1:13" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A122" s="52" t="s">
+      <c r="B122" s="1"/>
+    </row>
+    <row r="123" spans="1:13" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A123" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="B122" s="1"/>
-    </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A124" s="51" t="s">
-        <v>132</v>
-      </c>
-      <c r="B124" s="8"/>
-      <c r="C124" s="15" t="s">
-        <v>133</v>
-      </c>
+      <c r="B123" s="1"/>
     </row>
     <row r="125" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A125" s="51" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B125" s="8"/>
       <c r="C125" s="15" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A126" s="51" t="s">
+        <v>134</v>
+      </c>
+      <c r="B126" s="8"/>
+      <c r="C126" s="15" t="s">
         <v>135</v>
       </c>
     </row>
@@ -5346,6 +5925,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010021AB849DB9524648A8F6CDAE5A42EE85" ma:contentTypeVersion="54" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5cf342e325584cfc73779b32cd8516cb">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="7b6a70c9-bad9-43e8-985b-3d2ca80c98eb" xmlns:ns3="06fec347-a373-485e-bb4f-f611040a1dd3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="97bec9e280156beb57af844d85b9963b" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5745,15 +6333,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C64067D8-2529-40F8-873F-7DCFF29E6C0A}">
   <ds:schemaRefs>
@@ -5773,6 +6352,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5D2ED08-240E-422E-815D-BA2AE63D0B29}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B271E1E9-4B5A-43C8-93E9-EF9A1A456C27}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5790,12 +6377,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5D2ED08-240E-422E-815D-BA2AE63D0B29}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ajustes slider tolltip, botón , móvil etc.
</commit_message>
<xml_diff>
--- a/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2_15-10-2026.xlsx
+++ b/src/Documentacion/BIS011APPSY-SeguimientoPlanTrabajoDesaHERRIZ-v2_15-10-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sgantolin\BiscaytikApp_node-modules-incluido\src\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6676DE-052C-4BF0-98D8-190CF8C7583E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D819444C-89CB-4A16-988E-E7D216D3E791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="284">
   <si>
     <t>HITO</t>
   </si>
@@ -839,28 +839,55 @@
     <t>80% Finalizado. 1ra prueba hecha.</t>
   </si>
   <si>
-    <t xml:space="preserve">
-I de información es un tooltip https://getbootstrap.com/docs/5.0/components/tooltips/ cualquier cosa nos comentáis pues tenemos el código en local
-La i he visto que tenía una BKTT-Icon dentro de otro BKTT-Icon. El padre debería ser BKTT-Button btn btn-link. I si el icono de dentro es &lt;i class="fa-regular fa-info"&gt;&lt;/i&gt; en vez del cicle fenomenal
-Las a's que entiendo que son los botones de CTA, deberían de tener la siguiente class BKTT-Button btn btn-primary. Sobre todo BKTT-Button</t>
-  </si>
-  <si>
-    <t>Muy dificil rojoy media amarillo</t>
-  </si>
-  <si>
     <t>3.1 HOME http://turi.santurtzi.com/es-es/Paginas/Default2.aspx</t>
   </si>
   <si>
-    <t>SUMMARYLINKSLIDER2026</t>
-  </si>
-  <si>
-    <t>SUMMARYLINK2026</t>
-  </si>
-  <si>
     <t>SUMMARYLINKSLIDER2026 (15/10/2026)</t>
   </si>
   <si>
     <t>SUMMARYLINK2026 (15/10/2026)</t>
+  </si>
+  <si>
+    <t>Sin comenzar (no prioritario)</t>
+  </si>
+  <si>
+    <t>A la espera modificaciones y definición con DESA. Opción bg transparente?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condicionado a que todos los compoenntes estén "finalizados" sin test wpz. </t>
+  </si>
+  <si>
+    <t>Confirmar que se muestra 3 en vez de 4 por falta de contenido</t>
+  </si>
+  <si>
+    <t>necesaria opción columna o row</t>
+  </si>
+  <si>
+    <t>dropdown submenú https://getbootstrap.com/docs/4.0/components/dropdowns/</t>
+  </si>
+  <si>
+    <t>incluir Servicios?</t>
+  </si>
+  <si>
+    <t>Incluir algún dato más?</t>
+  </si>
+  <si>
+    <t>SUMMARYLINK2026 (destacados)</t>
+  </si>
+  <si>
+    <t>SUMMARYLINKSLIDER2026 (cards slider)</t>
+  </si>
+  <si>
+    <t>Propuesta de nav en email</t>
+  </si>
+  <si>
+    <t>bis anterior</t>
+  </si>
+  <si>
+    <t>no prioritario</t>
+  </si>
+  <si>
+    <t>Pendiente edición padre</t>
   </si>
 </sst>
 </file>
@@ -871,7 +898,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1026,6 +1053,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1185,7 +1220,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1354,6 +1389,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2158,7 +2196,7 @@
       <c r="AK14" s="19"/>
       <c r="AL14" s="19"/>
     </row>
-    <row r="15" spans="1:38" ht="57.6" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:38" ht="115.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>33</v>
       </c>
@@ -2194,11 +2232,15 @@
       </c>
       <c r="AH15" s="19"/>
       <c r="AI15" s="19"/>
-      <c r="AJ15" s="43" t="s">
-        <v>247</v>
-      </c>
-      <c r="AK15" s="19"/>
-      <c r="AL15" s="19"/>
+      <c r="AJ15" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK15" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="AL15" s="63" t="s">
+        <v>280</v>
+      </c>
     </row>
     <row r="16" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A16" s="13" t="s">
@@ -2906,7 +2948,7 @@
       <c r="AK34" s="19"/>
       <c r="AL34" s="19"/>
     </row>
-    <row r="35" spans="1:38" ht="409.6" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:38" ht="86.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A35" s="13" t="s">
         <v>177</v>
       </c>
@@ -2969,15 +3011,11 @@
       <c r="AI35" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="AJ35" s="44" t="s">
-        <v>166</v>
-      </c>
-      <c r="AK35" s="19" t="s">
-        <v>267</v>
-      </c>
-      <c r="AL35" s="19" t="s">
-        <v>232</v>
-      </c>
+      <c r="AJ35" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK35" s="19"/>
+      <c r="AL35" s="19"/>
     </row>
     <row r="36" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A36" s="13" t="s">
@@ -3057,7 +3095,7 @@
       <c r="AK37" s="19"/>
       <c r="AL37" s="19"/>
     </row>
-    <row r="38" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:38" ht="28.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A38" s="13" t="s">
         <v>56</v>
       </c>
@@ -3080,7 +3118,9 @@
       <c r="AG38" s="19"/>
       <c r="AH38" s="19"/>
       <c r="AI38" s="19"/>
-      <c r="AJ38" s="19"/>
+      <c r="AJ38" s="47" t="s">
+        <v>270</v>
+      </c>
       <c r="AK38" s="19"/>
       <c r="AL38" s="19"/>
     </row>
@@ -3314,7 +3354,7 @@
     </row>
     <row r="45" spans="1:38" ht="72" x14ac:dyDescent="0.3">
       <c r="A45" s="50" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B45" s="16" t="s">
         <v>64</v>
@@ -3365,14 +3405,10 @@
         <v>263</v>
       </c>
       <c r="AJ45" s="44" t="s">
-        <v>262</v>
-      </c>
-      <c r="AK45" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="AL45" s="19" t="s">
-        <v>263</v>
-      </c>
+        <v>272</v>
+      </c>
+      <c r="AK45" s="19"/>
+      <c r="AL45" s="64"/>
     </row>
     <row r="46" spans="1:38" ht="28.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A46" s="19" t="s">
@@ -3430,12 +3466,10 @@
       <c r="AJ46" s="43" t="s">
         <v>165</v>
       </c>
-      <c r="AK46" s="19" t="s">
-        <v>210</v>
-      </c>
+      <c r="AK46" s="19"/>
       <c r="AL46" s="19"/>
     </row>
-    <row r="47" spans="1:38" ht="43.2" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A47" s="19" t="s">
         <v>67</v>
       </c>
@@ -3491,9 +3525,7 @@
       <c r="AJ47" s="43" t="s">
         <v>165</v>
       </c>
-      <c r="AK47" s="63" t="s">
-        <v>268</v>
-      </c>
+      <c r="AK47" s="19"/>
       <c r="AL47" s="19"/>
     </row>
     <row r="48" spans="1:38" ht="86.4" outlineLevel="2" x14ac:dyDescent="0.3">
@@ -3552,15 +3584,13 @@
         <v>186</v>
       </c>
       <c r="AI48" s="19"/>
-      <c r="AJ48" s="45" t="s">
-        <v>167</v>
-      </c>
-      <c r="AK48" s="19" t="s">
+      <c r="AJ48" s="47" t="s">
         <v>186</v>
       </c>
+      <c r="AK48" s="19"/>
       <c r="AL48" s="19"/>
     </row>
-    <row r="49" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:38" ht="86.4" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A49" s="32" t="s">
         <v>254</v>
       </c>
@@ -3577,10 +3607,12 @@
       </c>
       <c r="AH49" s="19"/>
       <c r="AI49" s="19"/>
-      <c r="AJ49" s="45" t="s">
-        <v>167</v>
-      </c>
-      <c r="AK49" s="19"/>
+      <c r="AJ49" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK49" s="63" t="s">
+        <v>273</v>
+      </c>
       <c r="AL49" s="19"/>
     </row>
     <row r="50" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
@@ -3603,10 +3635,12 @@
       </c>
       <c r="AH50" s="19"/>
       <c r="AI50" s="19"/>
-      <c r="AJ50" s="45" t="s">
-        <v>167</v>
-      </c>
-      <c r="AK50" s="19"/>
+      <c r="AJ50" s="43" t="s">
+        <v>165</v>
+      </c>
+      <c r="AK50" s="63" t="s">
+        <v>281</v>
+      </c>
       <c r="AL50" s="19"/>
     </row>
     <row r="51" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
@@ -3629,13 +3663,13 @@
       </c>
       <c r="AH51" s="19"/>
       <c r="AI51" s="19"/>
-      <c r="AJ51" s="45" t="s">
-        <v>167</v>
+      <c r="AJ51" s="43" t="s">
+        <v>165</v>
       </c>
       <c r="AK51" s="19"/>
       <c r="AL51" s="19"/>
     </row>
-    <row r="52" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:38" ht="57.6" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A52" s="32" t="s">
         <v>259</v>
       </c>
@@ -3655,13 +3689,15 @@
       </c>
       <c r="AH52" s="19"/>
       <c r="AI52" s="19"/>
-      <c r="AJ52" s="45" t="s">
-        <v>167</v>
-      </c>
-      <c r="AK52" s="19"/>
+      <c r="AJ52" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK52" s="63" t="s">
+        <v>274</v>
+      </c>
       <c r="AL52" s="19"/>
     </row>
-    <row r="53" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:38" ht="28.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A53" s="32" t="s">
         <v>257</v>
       </c>
@@ -3681,11 +3717,13 @@
       </c>
       <c r="AH53" s="19"/>
       <c r="AI53" s="19"/>
-      <c r="AJ53" s="45" t="s">
-        <v>167</v>
+      <c r="AJ53" s="44" t="s">
+        <v>166</v>
       </c>
       <c r="AK53" s="19"/>
-      <c r="AL53" s="19"/>
+      <c r="AL53" s="63" t="s">
+        <v>276</v>
+      </c>
     </row>
     <row r="54" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A54" s="32" t="s">
@@ -3707,13 +3745,13 @@
       </c>
       <c r="AH54" s="19"/>
       <c r="AI54" s="19"/>
-      <c r="AJ54" s="45" t="s">
-        <v>167</v>
+      <c r="AJ54" s="43" t="s">
+        <v>165</v>
       </c>
       <c r="AK54" s="19"/>
       <c r="AL54" s="19"/>
     </row>
-    <row r="55" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:38" ht="28.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A55" s="32" t="s">
         <v>258</v>
       </c>
@@ -3733,11 +3771,13 @@
       </c>
       <c r="AH55" s="19"/>
       <c r="AI55" s="19"/>
-      <c r="AJ55" s="45" t="s">
-        <v>167</v>
+      <c r="AJ55" s="43" t="s">
+        <v>165</v>
       </c>
       <c r="AK55" s="19"/>
-      <c r="AL55" s="19"/>
+      <c r="AL55" s="63" t="s">
+        <v>277</v>
+      </c>
     </row>
     <row r="56" spans="1:38" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A56" s="32" t="s">
@@ -3759,13 +3799,13 @@
       </c>
       <c r="AH56" s="19"/>
       <c r="AI56" s="19"/>
-      <c r="AJ56" s="46" t="s">
-        <v>168</v>
+      <c r="AJ56" s="43" t="s">
+        <v>165</v>
       </c>
       <c r="AK56" s="19"/>
       <c r="AL56" s="19"/>
     </row>
-    <row r="57" spans="1:38" ht="72" outlineLevel="2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:38" ht="115.2" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="A57" s="33" t="s">
         <v>171</v>
       </c>
@@ -3822,7 +3862,7 @@
         <v>246</v>
       </c>
       <c r="AK57" s="55" t="s">
-        <v>241</v>
+        <v>271</v>
       </c>
       <c r="AL57" s="19"/>
     </row>
@@ -4711,7 +4751,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="85" spans="1:38" ht="100.8" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:38" ht="72" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A85" s="13" t="s">
         <v>88</v>
       </c>
@@ -4903,7 +4943,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="89" spans="1:38" ht="100.8" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:38" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A89" s="30" t="s">
         <v>95</v>
       </c>
@@ -5351,7 +5391,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="98" spans="1:38" ht="86.4" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:38" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>109</v>
       </c>
@@ -5400,7 +5440,7 @@
         <v>249</v>
       </c>
       <c r="AJ98" s="43" t="s">
-        <v>245</v>
+        <v>165</v>
       </c>
       <c r="AK98" s="19"/>
       <c r="AL98" s="19" t="s">
@@ -5409,10 +5449,10 @@
     </row>
     <row r="99" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="C99" s="16" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="D99" s="13"/>
       <c r="E99" s="6"/>
@@ -5429,16 +5469,18 @@
       <c r="AG99" s="43"/>
       <c r="AH99" s="19"/>
       <c r="AI99" s="19"/>
-      <c r="AJ99" s="43"/>
+      <c r="AJ99" s="47" t="s">
+        <v>282</v>
+      </c>
       <c r="AK99" s="19"/>
       <c r="AL99" s="19"/>
     </row>
-    <row r="100" spans="1:38" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:38" ht="43.2" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="C100" s="16" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D100" s="13"/>
       <c r="E100" s="6"/>
@@ -5455,11 +5497,15 @@
       <c r="AG100" s="43"/>
       <c r="AH100" s="19"/>
       <c r="AI100" s="19"/>
-      <c r="AJ100" s="43"/>
-      <c r="AK100" s="19"/>
+      <c r="AJ100" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="AK100" s="63" t="s">
+        <v>283</v>
+      </c>
       <c r="AL100" s="19"/>
     </row>
-    <row r="101" spans="1:38" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:38" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A101" s="50" t="s">
         <v>223</v>
       </c>
@@ -5711,7 +5757,7 @@
       <c r="AK109" s="19"/>
       <c r="AL109" s="19"/>
     </row>
-    <row r="110" spans="1:38" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:38" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A110" s="50" t="s">
         <v>224</v>
       </c>

</xml_diff>